<commit_message>
Fixed issue when copying worksheets with headers and footers
</commit_message>
<xml_diff>
--- a/ClosedXML/ClosedXML/ClosedXML_Tests/Resource/Examples/Misc/CopyingWorksheets.xlsx
+++ b/ClosedXML/ClosedXML/ClosedXML_Tests/Resource/Examples/Misc/CopyingWorksheets.xlsx
@@ -1114,7 +1114,14 @@
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
-  <x:headerFooter/>
+  <x:headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="1" alignWithMargins="1">
+    <x:oddHeader/>
+    <x:oddFooter/>
+    <x:evenHeader/>
+    <x:evenFooter/>
+    <x:firstHeader/>
+    <x:firstFooter/>
+  </x:headerFooter>
   <x:tableParts count="3">
     <x:tablePart r:id="rId13"/>
     <x:tablePart r:id="rId14"/>
@@ -1223,7 +1230,14 @@
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
-  <x:headerFooter/>
+  <x:headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="1" alignWithMargins="1">
+    <x:oddHeader/>
+    <x:oddFooter/>
+    <x:evenHeader/>
+    <x:evenFooter/>
+    <x:firstHeader/>
+    <x:firstFooter/>
+  </x:headerFooter>
   <x:tableParts count="0"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Even more memory and performance improvements.
</commit_message>
<xml_diff>
--- a/ClosedXML/ClosedXML/ClosedXML_Tests/Resource/Examples/Misc/CopyingWorksheets.xlsx
+++ b/ClosedXML/ClosedXML/ClosedXML_Tests/Resource/Examples/Misc/CopyingWorksheets.xlsx
@@ -356,10 +356,10 @@
     <x:xf numFmtId="1" fontId="0" fillId="0" borderId="9" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="0" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="1" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
     <x:xf numFmtId="15" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="1" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="15" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="1">
@@ -454,11 +454,11 @@
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
     <x:xf numFmtId="15" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>

</xml_diff>